<commit_message>
fix: harden siparis excel template and export flow
</commit_message>
<xml_diff>
--- a/CamSistemWebArayuz/Assets/sablonStokYeni.xlsx
+++ b/CamSistemWebArayuz/Assets/sablonStokYeni.xlsx
@@ -1,36 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" ns1:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PİMEKS\05.12.2025 YEDEK\Cafer\CamSistem\CamSistem\CamSistemWebArayuz\Assets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8068C1B-4A6A-4CC5-9D14-65E5DF1F011B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="D:\PİMEKS\05.12.2025 YEDEK\Cafer\CamSistem\CamSistem\CamSistemWebArayuz\Assets\"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8068C1B-4A6A-4CC5-9D14-65E5DF1F011B}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" ns6:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sayfa1" sheetId="40" r:id="rId1"/>
+    <sheet name="Siparis" sheetId="40" ns7:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sayfa1!$A$1:$L$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <ns8:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
+    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns9:calcFeatures>
+        <ns9:feature name="microsoft.com:RD"/>
+        <ns9:feature name="microsoft.com:Single"/>
+        <ns9:feature name="microsoft.com:FV"/>
+        <ns9:feature name="microsoft.com:CNMTM"/>
+        <ns9:feature name="microsoft.com:LET_WF"/>
+      </ns9:calcFeatures>
     </ext>
   </extLst>
 </workbook>

</xml_diff>

<commit_message>
fix: strip richData/metadata from Excel template and improve error logging
</commit_message>
<xml_diff>
--- a/CamSistemWebArayuz/Assets/sablonStokYeni.xlsx
+++ b/CamSistemWebArayuz/Assets/sablonStokYeni.xlsx
@@ -34,28 +34,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </valueMetadata>
-</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -788,70 +766,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1139,9 +1053,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1">
-      <c r="A1" s="62" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A1" s="62"/>
       <c r="B1" s="63"/>
       <c r="C1" s="68" t="s">
         <v>14</v>

</xml_diff>